<commit_message>
G1 exact submission (scored 100%); respect hackathon 5-job limit
- submissions/G1_v1.csv: exact <Z_q> for all 30 Duke_G1_q circuits on
  BlueQubit's cpu device (0 credits). Uploaded to the G1 problem: score 100%
  (corr^2 = 1).
- runs/hidden_1.xlsx and runs/ledger.csv: G1 exact values and job records.
- runner: default max_in_flight = 5 (hackathon limit of 5 concurrent jobs per
  account); jobs refused with HACKATHON_PARALLEL_JOBS_LIMIT are retried instead
  of marked failed.
- tests: workbook setup may overwrite the test's copy, which now holds real data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/runs/hidden_1.xlsx
+++ b/runs/hidden_1.xlsx
@@ -7,6 +7,7 @@
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimates" sheetId="3" r:id="R692b76a15434439e"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs" sheetId="4" r:id="R1a71762bf4404427"/>
   </x:sheets>
+  <x:calcPr fullCalcOnLoad="1"/>
 </x:workbook>
 </file>
 
@@ -467,7 +468,11 @@
       <x:c r="A4" s="2" t="str">
         <x:v>Official circuit ID</x:v>
       </x:c>
-      <x:c r="B4" s="6"/>
+      <x:c r="B4" s="6" t="inlineStr">
+        <x:is>
+          <x:t>G1</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C4" s="2"/>
       <x:c r="D4" s="10" t="str">
         <x:v>Precision settings</x:v>
@@ -487,7 +492,9 @@
       <x:c r="A5" s="2" t="str">
         <x:v>Required qubits</x:v>
       </x:c>
-      <x:c r="B5" s="6"/>
+      <x:c r="B5" s="6" t="n">
+        <x:v>30</x:v>
+      </x:c>
       <x:c r="C5" s="2"/>
       <x:c r="D5" s="2" t="str">
         <x:v>MPS bond dimension χ</x:v>
@@ -1124,8 +1131,12 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="21"/>
-      <x:c r="B6" s="19"/>
+      <x:c r="A6" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B6" s="19" t="n">
+        <x:v>-0.0002501840465460624</x:v>
+      </x:c>
       <x:c r="C6" s="13" t="str">
         <x:f>IF(OR(COUNTA($A6)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A6,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A6,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A6,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A6,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1180,8 +1191,12 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="21"/>
-      <x:c r="B7" s="19"/>
+      <x:c r="A7" s="21" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B7" s="19" t="n">
+        <x:v>0.0014240241043009729</x:v>
+      </x:c>
       <x:c r="C7" s="13" t="str">
         <x:f>IF(OR(COUNTA($A7)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A7,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A7,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A7,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A7,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1236,8 +1251,12 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="21"/>
-      <x:c r="B8" s="19"/>
+      <x:c r="A8" s="21" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B8" s="19" t="n">
+        <x:v>-0.00044375747784213974</x:v>
+      </x:c>
       <x:c r="C8" s="13" t="str">
         <x:f>IF(OR(COUNTA($A8)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A8,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A8,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A8,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A8,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1292,8 +1311,12 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="21"/>
-      <x:c r="B9" s="19"/>
+      <x:c r="A9" s="21" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B9" s="19" t="n">
+        <x:v>-0.006020519256074278</x:v>
+      </x:c>
       <x:c r="C9" s="13" t="str">
         <x:f>IF(OR(COUNTA($A9)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A9,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A9,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A9,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A9,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1348,8 +1371,12 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="21"/>
-      <x:c r="B10" s="19"/>
+      <x:c r="A10" s="21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B10" s="19" t="n">
+        <x:v>-0.0002751088476296417</x:v>
+      </x:c>
       <x:c r="C10" s="13" t="str">
         <x:f>IF(OR(COUNTA($A10)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A10,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A10,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A10,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A10,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1404,8 +1431,12 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="21"/>
-      <x:c r="B11" s="19"/>
+      <x:c r="A11" s="21" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B11" s="19" t="n">
+        <x:v>-0.0010382802978458026</x:v>
+      </x:c>
       <x:c r="C11" s="13" t="str">
         <x:f>IF(OR(COUNTA($A11)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A11,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A11,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A11,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A11,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1460,8 +1491,12 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="21"/>
-      <x:c r="B12" s="19"/>
+      <x:c r="A12" s="21" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B12" s="19" t="n">
+        <x:v>-5.815893185304763e-05</x:v>
+      </x:c>
       <x:c r="C12" s="13" t="str">
         <x:f>IF(OR(COUNTA($A12)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A12,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A12,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A12,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A12,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1516,8 +1551,12 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="21"/>
-      <x:c r="B13" s="19"/>
+      <x:c r="A13" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B13" s="19" t="n">
+        <x:v>0.0002044213011354212</x:v>
+      </x:c>
       <x:c r="C13" s="13" t="str">
         <x:f>IF(OR(COUNTA($A13)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A13,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A13,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A13,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A13,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1572,8 +1611,12 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="21"/>
-      <x:c r="B14" s="19"/>
+      <x:c r="A14" s="21" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B14" s="19" t="n">
+        <x:v>0.00016644082205444978</x:v>
+      </x:c>
       <x:c r="C14" s="13" t="str">
         <x:f>IF(OR(COUNTA($A14)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A14,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A14,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A14,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A14,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1628,8 +1671,12 @@
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="21"/>
-      <x:c r="B15" s="19"/>
+      <x:c r="A15" s="21" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B15" s="19" t="n">
+        <x:v>-0.000373459593607635</x:v>
+      </x:c>
       <x:c r="C15" s="13" t="str">
         <x:f>IF(OR(COUNTA($A15)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A15,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A15,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A15,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A15,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1684,8 +1731,12 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="21"/>
-      <x:c r="B16" s="19"/>
+      <x:c r="A16" s="21" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B16" s="19" t="n">
+        <x:v>0.0008473618512345215</x:v>
+      </x:c>
       <x:c r="C16" s="13" t="str">
         <x:f>IF(OR(COUNTA($A16)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A16,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A16,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A16,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A16,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1740,8 +1791,12 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="21"/>
-      <x:c r="B17" s="19"/>
+      <x:c r="A17" s="21" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B17" s="19" t="n">
+        <x:v>-8.081318254257477e-05</x:v>
+      </x:c>
       <x:c r="C17" s="13" t="str">
         <x:f>IF(OR(COUNTA($A17)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A17,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A17,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A17,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A17,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1796,8 +1851,12 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="21"/>
-      <x:c r="B18" s="19"/>
+      <x:c r="A18" s="21" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B18" s="19" t="n">
+        <x:v>-0.003098436594223144</x:v>
+      </x:c>
       <x:c r="C18" s="13" t="str">
         <x:f>IF(OR(COUNTA($A18)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A18,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A18,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A18,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A18,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1852,8 +1911,12 @@
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="21"/>
-      <x:c r="B19" s="19"/>
+      <x:c r="A19" s="21" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B19" s="19" t="n">
+        <x:v>-0.0035378557007047784</x:v>
+      </x:c>
       <x:c r="C19" s="13" t="str">
         <x:f>IF(OR(COUNTA($A19)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A19,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A19,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A19,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A19,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1908,8 +1971,12 @@
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="21"/>
-      <x:c r="B20" s="19"/>
+      <x:c r="A20" s="21" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B20" s="19" t="n">
+        <x:v>-0.045039793461481854</x:v>
+      </x:c>
       <x:c r="C20" s="13" t="str">
         <x:f>IF(OR(COUNTA($A20)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A20,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A20,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A20,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A20,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1964,8 +2031,12 @@
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="21"/>
-      <x:c r="B21" s="19"/>
+      <x:c r="A21" s="21" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B21" s="19" t="n">
+        <x:v>-0.020074852421475862</x:v>
+      </x:c>
       <x:c r="C21" s="13" t="str">
         <x:f>IF(OR(COUNTA($A21)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A21,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A21,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A21,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A21,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -2020,8 +2091,12 @@
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="21"/>
-      <x:c r="B22" s="19"/>
+      <x:c r="A22" s="21" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B22" s="19" t="n">
+        <x:v>-0.022219678173102678</x:v>
+      </x:c>
       <x:c r="C22" s="13" t="str">
         <x:f>IF(OR(COUNTA($A22)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A22,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A22,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A22,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A22,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -2076,8 +2151,12 @@
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="21"/>
-      <x:c r="B23" s="19"/>
+      <x:c r="A23" s="21" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B23" s="19" t="n">
+        <x:v>-0.03485530573064188</x:v>
+      </x:c>
       <x:c r="C23" s="13" t="str">
         <x:f>IF(OR(COUNTA($A23)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A23,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A23,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A23,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A23,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -2132,8 +2211,12 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="21"/>
-      <x:c r="B24" s="19"/>
+      <x:c r="A24" s="21" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B24" s="19" t="n">
+        <x:v>-0.03542460693511112</x:v>
+      </x:c>
       <x:c r="C24" s="13" t="str">
         <x:f>IF(OR(COUNTA($A24)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A24,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A24,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A24,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A24,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -2188,8 +2271,12 @@
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="21"/>
-      <x:c r="B25" s="19"/>
+      <x:c r="A25" s="21" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B25" s="19" t="n">
+        <x:v>-0.019191333739257386</x:v>
+      </x:c>
       <x:c r="C25" s="13" t="str">
         <x:f>IF(OR(COUNTA($A25)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A25,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A25,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A25,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A25,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -2244,8 +2331,12 @@
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="21"/>
-      <x:c r="B26" s="19"/>
+      <x:c r="A26" s="21" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B26" s="19" t="n">
+        <x:v>0.08375820732718607</x:v>
+      </x:c>
       <x:c r="C26" s="13" t="str">
         <x:f>IF(OR(COUNTA($A26)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A26,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A26,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A26,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A26,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -2300,8 +2391,12 @@
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="21"/>
-      <x:c r="B27" s="19"/>
+      <x:c r="A27" s="21" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B27" s="19" t="n">
+        <x:v>0.043056811260367915</x:v>
+      </x:c>
       <x:c r="C27" s="13" t="str">
         <x:f>IF(OR(COUNTA($A27)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A27,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A27,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A27,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A27,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -2356,8 +2451,12 @@
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="21"/>
-      <x:c r="B28" s="19"/>
+      <x:c r="A28" s="21" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B28" s="19" t="n">
+        <x:v>0.34578834474200254</x:v>
+      </x:c>
       <x:c r="C28" s="13" t="str">
         <x:f>IF(OR(COUNTA($A28)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A28,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A28,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A28,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A28,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -2412,8 +2511,12 @@
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="21"/>
-      <x:c r="B29" s="19"/>
+      <x:c r="A29" s="21" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B29" s="19" t="n">
+        <x:v>0.4559366929310495</x:v>
+      </x:c>
       <x:c r="C29" s="13" t="str">
         <x:f>IF(OR(COUNTA($A29)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A29,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A29,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A29,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A29,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -2468,8 +2571,12 @@
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="21"/>
-      <x:c r="B30" s="19"/>
+      <x:c r="A30" s="21" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B30" s="19" t="n">
+        <x:v>0.8332052108095281</x:v>
+      </x:c>
       <x:c r="C30" s="13" t="str">
         <x:f>IF(OR(COUNTA($A30)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A30,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A30,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A30,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A30,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -2524,8 +2631,12 @@
       </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="21"/>
-      <x:c r="B31" s="19"/>
+      <x:c r="A31" s="21" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B31" s="19" t="n">
+        <x:v>0.7762299006387924</x:v>
+      </x:c>
       <x:c r="C31" s="13" t="str">
         <x:f>IF(OR(COUNTA($A31)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A31,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A31,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A31,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A31,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -2580,8 +2691,12 @@
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="21"/>
-      <x:c r="B32" s="19"/>
+      <x:c r="A32" s="21" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B32" s="19" t="n">
+        <x:v>0.8984446072353612</x:v>
+      </x:c>
       <x:c r="C32" s="13" t="str">
         <x:f>IF(OR(COUNTA($A32)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A32,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A32,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A32,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A32,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -2636,8 +2751,12 @@
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="21"/>
-      <x:c r="B33" s="19"/>
+      <x:c r="A33" s="21" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B33" s="19" t="n">
+        <x:v>0.8767869009276636</x:v>
+      </x:c>
       <x:c r="C33" s="13" t="str">
         <x:f>IF(OR(COUNTA($A33)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A33,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A33,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A33,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A33,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -2692,8 +2811,12 @@
       </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="21"/>
-      <x:c r="B34" s="19"/>
+      <x:c r="A34" s="21" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B34" s="19" t="n">
+        <x:v>0.9315943818989001</x:v>
+      </x:c>
       <x:c r="C34" s="13" t="str">
         <x:f>IF(OR(COUNTA($A34)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A34,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A34,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A34,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A34,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -2748,8 +2871,12 @@
       </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="21"/>
-      <x:c r="B35" s="19"/>
+      <x:c r="A35" s="21" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B35" s="19" t="n">
+        <x:v>0.9514353510985869</x:v>
+      </x:c>
       <x:c r="C35" s="13" t="str">
         <x:f>IF(OR(COUNTA($A35)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A35,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A35,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A35,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A35,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -18370,266 +18497,1024 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="6"/>
-      <x:c r="B5" s="6"/>
+      <x:c r="A5" s="6" t="inlineStr">
+        <x:is>
+          <x:t>W6RnxKDgZZKi19cV</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B5" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C5" s="6"/>
       <x:c r="D5" s="11"/>
       <x:c r="E5" s="6"/>
-      <x:c r="F5" s="6"/>
-      <x:c r="G5" s="6"/>
-      <x:c r="H5" s="7"/>
-      <x:c r="I5" s="7"/>
-      <x:c r="J5" s="6"/>
+      <x:c r="F5" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G5" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H5" s="7" t="n">
+        <x:v>68.686</x:v>
+      </x:c>
+      <x:c r="I5" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 26883484649eba8a4d42</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="6"/>
-      <x:c r="B6" s="6"/>
+      <x:c r="A6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>XwidDPx5kTlxGMZm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C6" s="6"/>
       <x:c r="D6" s="11"/>
       <x:c r="E6" s="6"/>
-      <x:c r="F6" s="6"/>
-      <x:c r="G6" s="6"/>
-      <x:c r="H6" s="7"/>
-      <x:c r="I6" s="7"/>
-      <x:c r="J6" s="6"/>
+      <x:c r="F6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G6" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H6" s="7" t="n">
+        <x:v>62.502</x:v>
+      </x:c>
+      <x:c r="I6" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner c957bdd9d8fa0f2aacfe</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="6"/>
-      <x:c r="B7" s="6"/>
+      <x:c r="A7" s="6" t="inlineStr">
+        <x:is>
+          <x:t>ojyXDgQxjkg497PW</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C7" s="6"/>
       <x:c r="D7" s="11"/>
       <x:c r="E7" s="6"/>
-      <x:c r="F7" s="6"/>
-      <x:c r="G7" s="6"/>
-      <x:c r="H7" s="7"/>
-      <x:c r="I7" s="7"/>
-      <x:c r="J7" s="6"/>
+      <x:c r="F7" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G7" s="6" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H7" s="7" t="n">
+        <x:v>64.809</x:v>
+      </x:c>
+      <x:c r="I7" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J7" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner ec4138ce8455e5958a86</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="6"/>
-      <x:c r="B8" s="6"/>
+      <x:c r="A8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>GISWTrfrCQIgOrWq</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C8" s="6"/>
       <x:c r="D8" s="11"/>
       <x:c r="E8" s="6"/>
-      <x:c r="F8" s="6"/>
-      <x:c r="G8" s="6"/>
-      <x:c r="H8" s="7"/>
-      <x:c r="I8" s="7"/>
-      <x:c r="J8" s="6"/>
+      <x:c r="F8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G8" s="6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H8" s="7" t="n">
+        <x:v>57.064</x:v>
+      </x:c>
+      <x:c r="I8" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 8c24ee5a013e9c4a367a</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="6"/>
-      <x:c r="B9" s="6"/>
+      <x:c r="A9" s="6" t="inlineStr">
+        <x:is>
+          <x:t>1Q9k8h8XiQYn2QkK</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C9" s="6"/>
       <x:c r="D9" s="11"/>
       <x:c r="E9" s="6"/>
-      <x:c r="F9" s="6"/>
-      <x:c r="G9" s="6"/>
-      <x:c r="H9" s="7"/>
-      <x:c r="I9" s="7"/>
-      <x:c r="J9" s="6"/>
+      <x:c r="F9" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G9" s="6" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H9" s="7" t="n">
+        <x:v>65.349</x:v>
+      </x:c>
+      <x:c r="I9" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 178feb3f8d646bc3c645</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="6"/>
-      <x:c r="B10" s="6"/>
+      <x:c r="A10" s="6" t="inlineStr">
+        <x:is>
+          <x:t>OBHGogpwdgCQ5usD</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C10" s="6"/>
       <x:c r="D10" s="11"/>
       <x:c r="E10" s="6"/>
-      <x:c r="F10" s="6"/>
-      <x:c r="G10" s="6"/>
-      <x:c r="H10" s="7"/>
-      <x:c r="I10" s="7"/>
-      <x:c r="J10" s="6"/>
+      <x:c r="F10" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G10" s="6" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H10" s="7" t="n">
+        <x:v>71.683</x:v>
+      </x:c>
+      <x:c r="I10" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J10" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner d0bf0d79edb2f32f9d3c</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="6"/>
-      <x:c r="B11" s="6"/>
+      <x:c r="A11" s="6" t="inlineStr">
+        <x:is>
+          <x:t>V64qARnJGCrudOL7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C11" s="6"/>
       <x:c r="D11" s="11"/>
       <x:c r="E11" s="6"/>
-      <x:c r="F11" s="6"/>
-      <x:c r="G11" s="6"/>
-      <x:c r="H11" s="7"/>
-      <x:c r="I11" s="7"/>
-      <x:c r="J11" s="6"/>
+      <x:c r="F11" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G11" s="6" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H11" s="7" t="n">
+        <x:v>69.766</x:v>
+      </x:c>
+      <x:c r="I11" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J11" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner a1ad3d094cc5b3a2da92</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="6"/>
-      <x:c r="B12" s="6"/>
+      <x:c r="A12" s="6" t="inlineStr">
+        <x:is>
+          <x:t>oBn5grgusICRZNS5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C12" s="6"/>
       <x:c r="D12" s="11"/>
       <x:c r="E12" s="6"/>
-      <x:c r="F12" s="6"/>
-      <x:c r="G12" s="6"/>
-      <x:c r="H12" s="7"/>
-      <x:c r="I12" s="7"/>
-      <x:c r="J12" s="6"/>
+      <x:c r="F12" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G12" s="6" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H12" s="7" t="n">
+        <x:v>69.771</x:v>
+      </x:c>
+      <x:c r="I12" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J12" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 0f1c3b4f9f057b474156</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="6"/>
-      <x:c r="B13" s="6"/>
+      <x:c r="A13" s="6" t="inlineStr">
+        <x:is>
+          <x:t>jAFkvoA6IniilhXb</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C13" s="6"/>
       <x:c r="D13" s="11"/>
       <x:c r="E13" s="6"/>
-      <x:c r="F13" s="6"/>
-      <x:c r="G13" s="6"/>
-      <x:c r="H13" s="7"/>
-      <x:c r="I13" s="7"/>
-      <x:c r="J13" s="6"/>
+      <x:c r="F13" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G13" s="6" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H13" s="7" t="n">
+        <x:v>70.168</x:v>
+      </x:c>
+      <x:c r="I13" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J13" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner f85b7941dde431f79240</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="6"/>
-      <x:c r="B14" s="6"/>
+      <x:c r="A14" s="6" t="inlineStr">
+        <x:is>
+          <x:t>YiJe7ztq5vb6q0Mp</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C14" s="6"/>
       <x:c r="D14" s="11"/>
       <x:c r="E14" s="6"/>
-      <x:c r="F14" s="6"/>
-      <x:c r="G14" s="6"/>
-      <x:c r="H14" s="7"/>
-      <x:c r="I14" s="7"/>
-      <x:c r="J14" s="6"/>
+      <x:c r="F14" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G14" s="6" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H14" s="7" t="n">
+        <x:v>57.255</x:v>
+      </x:c>
+      <x:c r="I14" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J14" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 66de0da68e08e527ae25</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="6"/>
-      <x:c r="B15" s="6"/>
+      <x:c r="A15" s="6" t="inlineStr">
+        <x:is>
+          <x:t>6HcBXi5YMIFHmnIj</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C15" s="6"/>
       <x:c r="D15" s="11"/>
       <x:c r="E15" s="6"/>
-      <x:c r="F15" s="6"/>
-      <x:c r="G15" s="6"/>
-      <x:c r="H15" s="7"/>
-      <x:c r="I15" s="7"/>
-      <x:c r="J15" s="6"/>
+      <x:c r="F15" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G15" s="6" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H15" s="7" t="n">
+        <x:v>79.708</x:v>
+      </x:c>
+      <x:c r="I15" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J15" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 2f9b30db911ccd11cb9d</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="6"/>
-      <x:c r="B16" s="6"/>
+      <x:c r="A16" s="6" t="inlineStr">
+        <x:is>
+          <x:t>jJYWbtlne4KKS1aI</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C16" s="6"/>
       <x:c r="D16" s="11"/>
       <x:c r="E16" s="6"/>
-      <x:c r="F16" s="6"/>
-      <x:c r="G16" s="6"/>
-      <x:c r="H16" s="7"/>
-      <x:c r="I16" s="7"/>
-      <x:c r="J16" s="6"/>
+      <x:c r="F16" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G16" s="6" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H16" s="7" t="n">
+        <x:v>73.992</x:v>
+      </x:c>
+      <x:c r="I16" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J16" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner bae88c9fcd0c913f7300</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="6"/>
-      <x:c r="B17" s="6"/>
+      <x:c r="A17" s="6" t="inlineStr">
+        <x:is>
+          <x:t>x7V4njirlt7QWJ3V</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C17" s="6"/>
       <x:c r="D17" s="11"/>
       <x:c r="E17" s="6"/>
-      <x:c r="F17" s="6"/>
-      <x:c r="G17" s="6"/>
-      <x:c r="H17" s="7"/>
-      <x:c r="I17" s="7"/>
-      <x:c r="J17" s="6"/>
+      <x:c r="F17" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G17" s="6" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H17" s="7" t="n">
+        <x:v>68.787</x:v>
+      </x:c>
+      <x:c r="I17" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J17" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner ae78b042a1706222ec46</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="6"/>
-      <x:c r="B18" s="6"/>
+      <x:c r="A18" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Ofd8InoDWdzjMAMN</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C18" s="6"/>
       <x:c r="D18" s="11"/>
       <x:c r="E18" s="6"/>
-      <x:c r="F18" s="6"/>
-      <x:c r="G18" s="6"/>
-      <x:c r="H18" s="7"/>
-      <x:c r="I18" s="7"/>
-      <x:c r="J18" s="6"/>
+      <x:c r="F18" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G18" s="6" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="H18" s="7" t="n">
+        <x:v>57.984</x:v>
+      </x:c>
+      <x:c r="I18" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J18" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 3b030396ae20a3f459af</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="6"/>
-      <x:c r="B19" s="6"/>
+      <x:c r="A19" s="6" t="inlineStr">
+        <x:is>
+          <x:t>vgtq0xUxYCbYlZQG</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C19" s="6"/>
       <x:c r="D19" s="11"/>
       <x:c r="E19" s="6"/>
-      <x:c r="F19" s="6"/>
-      <x:c r="G19" s="6"/>
-      <x:c r="H19" s="7"/>
-      <x:c r="I19" s="7"/>
-      <x:c r="J19" s="6"/>
+      <x:c r="F19" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G19" s="6" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H19" s="7" t="n">
+        <x:v>58.386</x:v>
+      </x:c>
+      <x:c r="I19" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J19" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 6bf22169e26dbcaa584f</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="6"/>
-      <x:c r="B20" s="6"/>
+      <x:c r="A20" s="6" t="inlineStr">
+        <x:is>
+          <x:t>ZvvpXGUQP7CiOkzm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B20" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C20" s="6"/>
       <x:c r="D20" s="11"/>
       <x:c r="E20" s="6"/>
-      <x:c r="F20" s="6"/>
-      <x:c r="G20" s="6"/>
-      <x:c r="H20" s="7"/>
-      <x:c r="I20" s="7"/>
-      <x:c r="J20" s="6"/>
+      <x:c r="F20" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G20" s="6" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H20" s="7" t="n">
+        <x:v>78.033</x:v>
+      </x:c>
+      <x:c r="I20" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J20" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 277036aa1808d80f185f</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="21">
+      <x:c r="A21" t="inlineStr">
+        <x:is>
+          <x:t>RI1QjtifW6witQm3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B21" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21"/>
       <x:c r="D21" s="23"/>
-      <x:c r="H21" s="25"/>
-      <x:c r="I21" s="25"/>
+      <x:c r="E21"/>
+      <x:c r="F21" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G21" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="H21" s="25" t="n">
+        <x:v>64.555</x:v>
+      </x:c>
+      <x:c r="I21" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J21" t="inlineStr">
+        <x:is>
+          <x:t>runner 8950f0d1032b8720a72c</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="22">
+      <x:c r="A22" t="inlineStr">
+        <x:is>
+          <x:t>ciyPRzUyqLzY4ZJk</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B22" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22"/>
       <x:c r="D22" s="23"/>
-      <x:c r="H22" s="25"/>
-      <x:c r="I22" s="25"/>
+      <x:c r="E22"/>
+      <x:c r="F22" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G22" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="H22" s="25" t="n">
+        <x:v>57.087</x:v>
+      </x:c>
+      <x:c r="I22" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J22" t="inlineStr">
+        <x:is>
+          <x:t>runner a39d3a45363440739f57</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="23">
+      <x:c r="A23" t="inlineStr">
+        <x:is>
+          <x:t>GpN8Ugmh47AblPIN</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B23" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23"/>
       <x:c r="D23" s="23"/>
-      <x:c r="H23" s="25"/>
-      <x:c r="I23" s="25"/>
+      <x:c r="E23"/>
+      <x:c r="F23" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G23" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="H23" s="25" t="n">
+        <x:v>55.601</x:v>
+      </x:c>
+      <x:c r="I23" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J23" t="inlineStr">
+        <x:is>
+          <x:t>runner 54fd2484878ca38a62c4</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="24">
+      <x:c r="A24" t="inlineStr">
+        <x:is>
+          <x:t>OjcRynZujj9bi1JL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B24" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24"/>
       <x:c r="D24" s="23"/>
-      <x:c r="H24" s="25"/>
-      <x:c r="I24" s="25"/>
+      <x:c r="E24"/>
+      <x:c r="F24" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G24" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="H24" s="25" t="n">
+        <x:v>61.943</x:v>
+      </x:c>
+      <x:c r="I24" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J24" t="inlineStr">
+        <x:is>
+          <x:t>runner 46f5973e034fe3dd25fd</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="25">
+      <x:c r="A25" t="inlineStr">
+        <x:is>
+          <x:t>M9Yh3iot7G1983MX</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25"/>
       <x:c r="D25" s="23"/>
-      <x:c r="H25" s="25"/>
-      <x:c r="I25" s="25"/>
+      <x:c r="E25"/>
+      <x:c r="F25" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G25" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H25" s="25" t="n">
+        <x:v>54.652</x:v>
+      </x:c>
+      <x:c r="I25" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J25" t="inlineStr">
+        <x:is>
+          <x:t>runner 1fffff2201736ee597c4</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="26">
+      <x:c r="A26" t="inlineStr">
+        <x:is>
+          <x:t>9hP6o0yf8Qucz1G1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B26" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C26"/>
       <x:c r="D26" s="23"/>
-      <x:c r="H26" s="25"/>
-      <x:c r="I26" s="25"/>
+      <x:c r="E26"/>
+      <x:c r="F26" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G26" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H26" s="25" t="n">
+        <x:v>66.505</x:v>
+      </x:c>
+      <x:c r="I26" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J26" t="inlineStr">
+        <x:is>
+          <x:t>runner 3409f5de6c918987b0e2</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="27">
+      <x:c r="A27" t="inlineStr">
+        <x:is>
+          <x:t>BNx3CEpqYiyAvymm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B27" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C27"/>
       <x:c r="D27" s="23"/>
-      <x:c r="H27" s="25"/>
-      <x:c r="I27" s="25"/>
+      <x:c r="E27"/>
+      <x:c r="F27" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G27" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H27" s="25" t="n">
+        <x:v>67.228</x:v>
+      </x:c>
+      <x:c r="I27" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J27" t="inlineStr">
+        <x:is>
+          <x:t>runner 6641c278ea72884aef8c</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="28">
+      <x:c r="A28" t="inlineStr">
+        <x:is>
+          <x:t>EjyJwrEMlULvSVcO</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B28" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C28"/>
       <x:c r="D28" s="23"/>
-      <x:c r="H28" s="25"/>
-      <x:c r="I28" s="25"/>
+      <x:c r="E28"/>
+      <x:c r="F28" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G28" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H28" s="25" t="n">
+        <x:v>68.99</x:v>
+      </x:c>
+      <x:c r="I28" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J28" t="inlineStr">
+        <x:is>
+          <x:t>runner 8e7406482afffeacd905</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="29">
+      <x:c r="A29" t="inlineStr">
+        <x:is>
+          <x:t>TWb5RbiHJyoju2pt</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B29" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C29"/>
       <x:c r="D29" s="23"/>
-      <x:c r="H29" s="25"/>
-      <x:c r="I29" s="25"/>
+      <x:c r="E29"/>
+      <x:c r="F29" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G29" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H29" s="25" t="n">
+        <x:v>72.731</x:v>
+      </x:c>
+      <x:c r="I29" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J29" t="inlineStr">
+        <x:is>
+          <x:t>runner 1a8e5b2edeb01a5fd537</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="30">
+      <x:c r="A30" t="inlineStr">
+        <x:is>
+          <x:t>pUPV2rZIWoTpyOIX</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B30" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C30"/>
       <x:c r="D30" s="23"/>
-      <x:c r="H30" s="25"/>
-      <x:c r="I30" s="25"/>
+      <x:c r="E30"/>
+      <x:c r="F30" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G30" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="H30" s="25" t="n">
+        <x:v>73.536</x:v>
+      </x:c>
+      <x:c r="I30" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J30" t="inlineStr">
+        <x:is>
+          <x:t>runner b57f3a850ca811177a60</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="31">
+      <x:c r="A31" t="inlineStr">
+        <x:is>
+          <x:t>d8pQMdSejoYOvKgr</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B31" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C31"/>
       <x:c r="D31" s="23"/>
-      <x:c r="H31" s="25"/>
-      <x:c r="I31" s="25"/>
+      <x:c r="E31"/>
+      <x:c r="F31" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G31" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="H31" s="25" t="n">
+        <x:v>64.629</x:v>
+      </x:c>
+      <x:c r="I31" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J31" t="inlineStr">
+        <x:is>
+          <x:t>runner 4b3dfb7513979bc37afa</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="32">
+      <x:c r="A32" t="inlineStr">
+        <x:is>
+          <x:t>NjeORq7QmY3Au5Nk</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B32" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C32"/>
       <x:c r="D32" s="23"/>
-      <x:c r="H32" s="25"/>
-      <x:c r="I32" s="25"/>
+      <x:c r="E32"/>
+      <x:c r="F32" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G32" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H32" s="25" t="n">
+        <x:v>57.98</x:v>
+      </x:c>
+      <x:c r="I32" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J32" t="inlineStr">
+        <x:is>
+          <x:t>runner f1c547220151e8b37021</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="33">
+      <x:c r="A33" t="inlineStr">
+        <x:is>
+          <x:t>7v0hu2m2PN3gGsYQ</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B33" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C33"/>
       <x:c r="D33" s="23"/>
-      <x:c r="H33" s="25"/>
-      <x:c r="I33" s="25"/>
+      <x:c r="E33"/>
+      <x:c r="F33" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G33" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="H33" s="25" t="n">
+        <x:v>69.283</x:v>
+      </x:c>
+      <x:c r="I33" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J33" t="inlineStr">
+        <x:is>
+          <x:t>runner 054ffd14aef8c18c24ca</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="34">
+      <x:c r="A34" t="inlineStr">
+        <x:is>
+          <x:t>ER9Y1wOKkVu478uM</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B34" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C34"/>
       <x:c r="D34" s="23"/>
-      <x:c r="H34" s="25"/>
-      <x:c r="I34" s="25"/>
+      <x:c r="E34"/>
+      <x:c r="F34" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G34" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="H34" s="25" t="n">
+        <x:v>67.377</x:v>
+      </x:c>
+      <x:c r="I34" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J34" t="inlineStr">
+        <x:is>
+          <x:t>runner c00e6953783eba758568</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="D35" s="23"/>

</xml_diff>